<commit_message>
feat(vazios): import the real empty-container worksheet
</commit_message>
<xml_diff>
--- a/public/templates/vazios-modelo.xlsx
+++ b/public/templates/vazios-modelo.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Vazios" sheetId="1" r:id="rId1"/>
+    <sheet name="Vazios EXP" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,61 +397,111 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Booking</v>
+        <v>CONTAINER</v>
       </c>
       <c r="B1" t="str">
-        <v>Container</v>
+        <v>BOOKING</v>
       </c>
       <c r="C1" t="str">
+        <v>VESSEL</v>
+      </c>
+      <c r="D1" t="str">
+        <v>VOYAGE</v>
+      </c>
+      <c r="E1" t="str">
+        <v>POD</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Current Status</v>
+      </c>
+      <c r="G1" t="str">
+        <v>HIGHLIGHTS</v>
+      </c>
+      <c r="H1" t="str">
+        <v>VISUAL CHECK</v>
+      </c>
+      <c r="I1" t="str">
+        <v>IMPORT EMPTY RETURN DATE</v>
+      </c>
+      <c r="J1" t="str">
+        <v>EMPTY GATE OUT</v>
+      </c>
+      <c r="K1" t="str">
+        <v>LOAD DATE</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ORDER No.</v>
+      </c>
+      <c r="M1" t="str">
+        <v>DEPOT</v>
+      </c>
+      <c r="N1" t="str">
+        <v>OT Handling %</v>
+      </c>
+      <c r="O1" t="str">
+        <v>OT Transporte %</v>
+      </c>
+      <c r="P1" t="str">
         <v>Tipo</v>
       </c>
-      <c r="D1" t="str">
-        <v>Data Movimentação</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Terminal Origem</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Destino</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Observações</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Porto Embarque</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Depot</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Material</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Bundle</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Transporte</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Hand-in</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Hand-out</v>
-      </c>
-      <c r="O1" t="str">
-        <v>OT Handling</v>
-      </c>
-      <c r="P1" t="str">
-        <v>OT Transporte</v>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ABCD1234567</v>
+      </c>
+      <c r="B2" t="str">
+        <v>BK-EXAMPLE</v>
+      </c>
+      <c r="C2" t="str">
+        <v>NAVIO</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0001</v>
+      </c>
+      <c r="E2" t="str">
+        <v>BRSSZ</v>
+      </c>
+      <c r="F2" t="str">
+        <v>EMPTY</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>NO</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v>OS-EXAMPLE</v>
+      </c>
+      <c r="M2" t="str">
+        <v>DEPOT-A</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2" t="str">
+        <v>40HC</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>